<commit_message>
Verify trainer and artifact guidebook lists against game data
Trainer list: every named teacher matched against NPCData, 2DEvents,
MapStats, Teacher topics and zzMAW_MoveTrainers.lua. Adds Jacques Kohl
and Rexella, fixes house and map names, repairs source hyperlinks and
flags PDF-only Grandmaster claims as "im Spiel prüfen".

Artifact list (release tag 4.5): DPS recomputed from calcPowerVitality,
Vitality uses the weakest resistance, texts and dice checked against Lua
and ITEMS.txt, Ania Selving added, both sheets re-sorted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAW_Guidebook/MAW_MMMerge_4_5_Trainerliste_V3.xlsx
+++ b/MAW_Guidebook/MAW_MMMerge_4_5_Trainerliste_V3.xlsx
@@ -354,7 +354,7 @@
     <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="85" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -398,7 +398,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F2" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1023, Topic 1539).</x:v>
       </x:c>
       <x:c r="G2" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -421,7 +421,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F3" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #998, Topic 1539).</x:v>
       </x:c>
       <x:c r="G3" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -438,13 +438,13 @@
         <x:v>Caao Salem</x:v>
       </x:c>
       <x:c r="D4" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E4" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F4" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #965, Topic 1540).</x:v>
       </x:c>
       <x:c r="G4" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -461,16 +461,16 @@
         <x:v>Caao Salem</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E5" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F5" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G5" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
@@ -490,10 +490,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; NPC aus älteren Daten.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #852, Topic 1567).</x:v>
       </x:c>
       <x:c r="G6" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MMMerge-NPCData</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -513,7 +513,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #856, Topic 1567).</x:v>
       </x:c>
       <x:c r="G7" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -527,19 +527,19 @@
         <x:v>Meister</x:v>
       </x:c>
       <x:c r="C8" s="14" t="str">
-        <x:v>—</x:v>
+        <x:v>Jacques Kohl</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
-        <x:v>Free Haven</x:v>
+        <x:v>Frozen Highlands</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F8" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; Name offen.</x:v>
+        <x:v>Laut NPCData einziger Alchemy-Meister in Enroth (NPC #819, Topic 1568). MAW-PDF nennt Free Haven – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G8" s="22" t="str">
-        <x:v>MAW-PDF 4.5</x:v>
+        <x:v>MMMerge-NPCData</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -559,7 +559,7 @@
         <x:v>Castle Stromgard</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; Name offen.</x:v>
+        <x:v>Kein passender NPC in Enroth laut Spieldaten; Angabe nur laut MAW-PDF – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G9" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
@@ -582,7 +582,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; Trainername offen.</x:v>
+        <x:v>Kein passender NPC in Enroth laut Spieldaten; Angabe nur laut MAW-PDF – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G10" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
@@ -605,7 +605,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; Trainername offen.</x:v>
+        <x:v>Kein passender NPC in Enroth laut Spieldaten; Angabe nur laut MAW-PDF – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G11" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
@@ -628,7 +628,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; Trainername offen.</x:v>
+        <x:v>Kein passender NPC in Enroth laut Spieldaten; Angabe nur laut MAW-PDF – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G12" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
@@ -651,10 +651,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; NPC aus älteren Daten.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #880, Topic 1571).</x:v>
       </x:c>
       <x:c r="G13" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MMMerge-NPCData</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
@@ -674,10 +674,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; NPC aus älteren Daten.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #933, Topic 1571).</x:v>
       </x:c>
       <x:c r="G14" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MMMerge-NPCData</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
@@ -697,10 +697,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; NPC aus älteren Daten.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #809, Topic 1572).</x:v>
       </x:c>
       <x:c r="G15" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MMMerge-NPCData</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
@@ -720,10 +720,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
-        <x:v>MAW-PDF bestätigt Lehrort; NPC aus älteren Daten.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G16" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
@@ -743,7 +743,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #927, Topic 1519).</x:v>
       </x:c>
       <x:c r="G17" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -766,7 +766,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #946, Topic 1519).</x:v>
       </x:c>
       <x:c r="G18" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -789,10 +789,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Altname nicht belegbar; Trainer noch offen.</x:v>
+        <x:v>Kein passender NPC in Enroth laut Spieldaten; Angabe nur laut MAW-PDF – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G19" s="22" t="str">
-        <x:v>MMMerge-NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
@@ -812,10 +812,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Altname nicht belegbar; Trainer noch offen.</x:v>
+        <x:v>Kein passender NPC in Enroth laut Spieldaten; Angabe nur laut MAW-PDF – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G20" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
@@ -829,13 +829,13 @@
         <x:v>Pat Skylark</x:v>
       </x:c>
       <x:c r="D21" s="22" t="str">
-        <x:v>Eel-Infested Waters</x:v>
+        <x:v>Eel Infested Waters</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #891, Topic 1527).</x:v>
       </x:c>
       <x:c r="G21" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -858,7 +858,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #970, Topic 1527).</x:v>
       </x:c>
       <x:c r="G22" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -872,7 +872,7 @@
         <x:v>Meister</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>—</x:v>
+        <x:v>Rexella</x:v>
       </x:c>
       <x:c r="D23" s="22" t="str">
         <x:v>Paradise Valley</x:v>
@@ -881,7 +881,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Altname nicht belegbar; Trainer noch offen.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #915, Topic 1528).</x:v>
       </x:c>
       <x:c r="G23" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -895,7 +895,7 @@
         <x:v>Großmeister</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>—</x:v>
+        <x:v>Rexella</x:v>
       </x:c>
       <x:c r="D24" s="22" t="str">
         <x:v>Paradise Valley</x:v>
@@ -904,10 +904,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Altname nicht belegbar; Trainer noch offen.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G24" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
@@ -927,7 +927,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #820, Topic 1549).</x:v>
       </x:c>
       <x:c r="G25" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -950,7 +950,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1010, Topic 1549).</x:v>
       </x:c>
       <x:c r="G26" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -973,7 +973,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #840, Topic 1550).</x:v>
       </x:c>
       <x:c r="G27" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -996,10 +996,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G28" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
@@ -1019,7 +1019,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #864, Topic 1561).</x:v>
       </x:c>
       <x:c r="G29" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1042,7 +1042,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #847, Topic 1561).</x:v>
       </x:c>
       <x:c r="G30" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1065,7 +1065,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #972, Topic 1562).</x:v>
       </x:c>
       <x:c r="G31" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1088,10 +1088,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G32" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
@@ -1111,7 +1111,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #884, Topic 1523).</x:v>
       </x:c>
       <x:c r="G33" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1134,7 +1134,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #878, Topic 1523).</x:v>
       </x:c>
       <x:c r="G34" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1157,7 +1157,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #973, Topic 1524).</x:v>
       </x:c>
       <x:c r="G35" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1180,10 +1180,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G36" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
@@ -1203,7 +1203,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #907, Topic 1533).</x:v>
       </x:c>
       <x:c r="G37" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1226,7 +1226,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #812, Topic 1533).</x:v>
       </x:c>
       <x:c r="G38" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1249,7 +1249,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #811, Topic 1534).</x:v>
       </x:c>
       <x:c r="G39" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1272,10 +1272,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G40" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
@@ -1295,7 +1295,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #827, Topic 1517).</x:v>
       </x:c>
       <x:c r="G41" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1318,7 +1318,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #988, Topic 1517).</x:v>
       </x:c>
       <x:c r="G42" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1341,7 +1341,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #995, Topic 1518).</x:v>
       </x:c>
       <x:c r="G43" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1364,10 +1364,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G44" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
@@ -1387,10 +1387,10 @@
         <x:v>Blades' End</x:v>
       </x:c>
       <x:c r="F45" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #175, Topic 363); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G45" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
@@ -1410,10 +1410,10 @@
         <x:v>Duelists' Edge</x:v>
       </x:c>
       <x:c r="F46" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #176, Topic 364); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G46" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
@@ -1433,10 +1433,10 @@
         <x:v>Duelists' Edge</x:v>
       </x:c>
       <x:c r="F47" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; MAW-PDF: Meister auch GM.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen. Echter GM-Lehrer: siehe Paradise Valley (nächste Zeile).</x:v>
       </x:c>
       <x:c r="G47" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
@@ -1453,13 +1453,13 @@
         <x:v>Paradise Valley</x:v>
       </x:c>
       <x:c r="E48" s="14" t="str">
-        <x:v>Tavern</x:v>
+        <x:v>The Last Chance (Taverne)</x:v>
       </x:c>
       <x:c r="F48" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #177, Topic 365); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G48" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
@@ -1479,7 +1479,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F49" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #982, Topic 1553).</x:v>
       </x:c>
       <x:c r="G49" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1502,7 +1502,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F50" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #881, Topic 1553).</x:v>
       </x:c>
       <x:c r="G50" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1525,7 +1525,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F51" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1040, Topic 1554).</x:v>
       </x:c>
       <x:c r="G51" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1548,10 +1548,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F52" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G52" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
@@ -1571,7 +1571,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F53" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #855, Topic 1569).</x:v>
       </x:c>
       <x:c r="G53" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1594,7 +1594,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F54" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #962, Topic 1569).</x:v>
       </x:c>
       <x:c r="G54" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1617,7 +1617,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F55" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #875, Topic 1570).</x:v>
       </x:c>
       <x:c r="G55" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1640,10 +1640,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F56" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G56" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
@@ -1663,10 +1663,10 @@
         <x:v>Buccaneers' Lair</x:v>
       </x:c>
       <x:c r="F57" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #530, Topic 396); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G57" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
@@ -1686,10 +1686,10 @@
         <x:v>Smugglers' Guild</x:v>
       </x:c>
       <x:c r="F58" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #531, Topic 397); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G58" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
@@ -1709,10 +1709,10 @@
         <x:v>Smugglers' Guild</x:v>
       </x:c>
       <x:c r="F59" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; MAW-PDF: Meister auch GM.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen. Echter GM-Lehrer: siehe Paradise Valley (nächste Zeile).</x:v>
       </x:c>
       <x:c r="G59" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
@@ -1729,13 +1729,13 @@
         <x:v>Paradise Valley</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>The Sparring Grounds</x:v>
+        <x:v>The Sparring Ground</x:v>
       </x:c>
       <x:c r="F60" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #532, Topic 398); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G60" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
@@ -1755,10 +1755,10 @@
         <x:v>Blades' End</x:v>
       </x:c>
       <x:c r="F61" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #178, Topic 369); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G61" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
@@ -1778,10 +1778,10 @@
         <x:v>Duelists' Edge</x:v>
       </x:c>
       <x:c r="F62" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #179, Topic 370); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G62" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
@@ -1801,10 +1801,10 @@
         <x:v>Duelists' Edge</x:v>
       </x:c>
       <x:c r="F63" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; MAW-PDF: Meister auch GM.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen. Echter GM-Lehrer: siehe Paradise Valley (nächste Zeile).</x:v>
       </x:c>
       <x:c r="G63" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
@@ -1821,13 +1821,13 @@
         <x:v>Paradise Valley</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>Tavern</x:v>
+        <x:v>The Last Chance (Taverne)</x:v>
       </x:c>
       <x:c r="F64" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #180, Topic 371); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G64" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
@@ -1847,7 +1847,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F65" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1021, Topic 1543).</x:v>
       </x:c>
       <x:c r="G65" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1870,7 +1870,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F66" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1001, Topic 1543).</x:v>
       </x:c>
       <x:c r="G66" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1893,7 +1893,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F67" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #894, Topic 1544).</x:v>
       </x:c>
       <x:c r="G67" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1916,10 +1916,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F68" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G68" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
@@ -1939,7 +1939,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F69" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #993, Topic 1537).</x:v>
       </x:c>
       <x:c r="G69" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1962,7 +1962,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F70" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #866, Topic 1537).</x:v>
       </x:c>
       <x:c r="G70" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -1979,13 +1979,13 @@
         <x:v>Jezebel</x:v>
       </x:c>
       <x:c r="D71" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F71" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #890, Topic 1538).</x:v>
       </x:c>
       <x:c r="G71" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2002,16 +2002,16 @@
         <x:v>Jezebel</x:v>
       </x:c>
       <x:c r="D72" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F72" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G72" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
@@ -2031,7 +2031,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F73" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #841, Topic 1555).</x:v>
       </x:c>
       <x:c r="G73" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2054,7 +2054,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F74" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #958, Topic 1555).</x:v>
       </x:c>
       <x:c r="G74" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2077,7 +2077,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F75" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #870, Topic 1556).</x:v>
       </x:c>
       <x:c r="G75" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2100,10 +2100,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F76" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G76" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
@@ -2123,10 +2123,10 @@
         <x:v>Buccaneers' Lair</x:v>
       </x:c>
       <x:c r="F77" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #536, Topic 402); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G77" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
@@ -2146,10 +2146,10 @@
         <x:v>Smugglers' Guild</x:v>
       </x:c>
       <x:c r="F78" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #537, Topic 403); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G78" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
@@ -2169,10 +2169,10 @@
         <x:v>Smugglers' Guild</x:v>
       </x:c>
       <x:c r="F79" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; MAW-PDF: Meister auch GM.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen. Echter GM-Lehrer: siehe Paradise Valley (nächste Zeile).</x:v>
       </x:c>
       <x:c r="G79" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
@@ -2189,13 +2189,13 @@
         <x:v>Paradise Valley</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>The Sparring Grounds</x:v>
+        <x:v>The Sparring Ground</x:v>
       </x:c>
       <x:c r="F80" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #538, Topic 404); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G80" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
@@ -2215,7 +2215,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F81" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #882, Topic 1531).</x:v>
       </x:c>
       <x:c r="G81" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2232,13 +2232,13 @@
         <x:v>Arthur O'Leery</x:v>
       </x:c>
       <x:c r="D82" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F82" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #981, Topic 1531).</x:v>
       </x:c>
       <x:c r="G82" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2261,7 +2261,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F83" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #830, Topic 1532).</x:v>
       </x:c>
       <x:c r="G83" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2284,10 +2284,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F84" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G84" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
@@ -2307,7 +2307,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F85" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #963, Topic 1551).</x:v>
       </x:c>
       <x:c r="G85" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2330,7 +2330,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F86" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #908, Topic 1551).</x:v>
       </x:c>
       <x:c r="G86" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2347,13 +2347,13 @@
         <x:v>Ki Lo Nee</x:v>
       </x:c>
       <x:c r="D87" s="22" t="str">
-        <x:v>Eel-Infested Waters</x:v>
+        <x:v>Eel Infested Waters</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F87" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1057, Topic 1552).</x:v>
       </x:c>
       <x:c r="G87" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2370,16 +2370,16 @@
         <x:v>Ki Lo Nee</x:v>
       </x:c>
       <x:c r="D88" s="22" t="str">
-        <x:v>Eel-Infested Waters</x:v>
+        <x:v>Eel Infested Waters</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F88" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G88" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
@@ -2399,7 +2399,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F89" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #876, Topic 1525).</x:v>
       </x:c>
       <x:c r="G89" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2422,7 +2422,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F90" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #974, Topic 1525).</x:v>
       </x:c>
       <x:c r="G90" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2445,7 +2445,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F91" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #874, Topic 1526).</x:v>
       </x:c>
       <x:c r="G91" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2468,10 +2468,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F92" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G92" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
@@ -2491,7 +2491,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F93" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #857, Topic 1563).</x:v>
       </x:c>
       <x:c r="G93" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2514,7 +2514,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F94" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #949, Topic 1563).</x:v>
       </x:c>
       <x:c r="G94" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2531,13 +2531,13 @@
         <x:v>Norio Ariganaka</x:v>
       </x:c>
       <x:c r="D95" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E95" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F95" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1014, Topic 1564).</x:v>
       </x:c>
       <x:c r="G95" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2554,16 +2554,16 @@
         <x:v>Norio Ariganaka</x:v>
       </x:c>
       <x:c r="D96" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E96" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F96" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G96" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
@@ -2583,7 +2583,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F97" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #867, Topic 1557).</x:v>
       </x:c>
       <x:c r="G97" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2606,7 +2606,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F98" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #957, Topic 1557).</x:v>
       </x:c>
       <x:c r="G98" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2629,7 +2629,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F99" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #814, Topic 1558).</x:v>
       </x:c>
       <x:c r="G99" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2652,10 +2652,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F100" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G100" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="28" customHeight="1">
@@ -2675,7 +2675,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F101" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #951, Topic 1547).</x:v>
       </x:c>
       <x:c r="G101" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2698,7 +2698,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F102" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #853, Topic 1547).</x:v>
       </x:c>
       <x:c r="G102" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2721,7 +2721,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F103" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #858, Topic 1548).</x:v>
       </x:c>
       <x:c r="G103" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2744,10 +2744,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F104" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G104" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="28" customHeight="1">
@@ -2767,7 +2767,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F105" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1015, Topic 1565).</x:v>
       </x:c>
       <x:c r="G105" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2790,7 +2790,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F106" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #910, Topic 1565).</x:v>
       </x:c>
       <x:c r="G106" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2813,7 +2813,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F107" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #842, Topic 1566).</x:v>
       </x:c>
       <x:c r="G107" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2836,10 +2836,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F108" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G108" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="28" customHeight="1">
@@ -2859,7 +2859,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F109" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #807, Topic 1535).</x:v>
       </x:c>
       <x:c r="G109" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2882,7 +2882,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F110" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #999, Topic 1535).</x:v>
       </x:c>
       <x:c r="G110" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2905,7 +2905,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F111" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #808, Topic 1536).</x:v>
       </x:c>
       <x:c r="G111" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -2928,10 +2928,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F112" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G112" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="28" customHeight="1">
@@ -2951,10 +2951,10 @@
         <x:v>Buccaneers' Lair</x:v>
       </x:c>
       <x:c r="F113" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #214, Topic 390); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G113" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="28" customHeight="1">
@@ -2974,10 +2974,10 @@
         <x:v>Smugglers' Guild</x:v>
       </x:c>
       <x:c r="F114" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #215, Topic 391); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G114" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="28" customHeight="1">
@@ -2997,10 +2997,10 @@
         <x:v>Smugglers' Guild</x:v>
       </x:c>
       <x:c r="F115" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; MAW-PDF: Meister auch GM.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen. Echter GM-Lehrer: siehe Paradise Valley (nächste Zeile).</x:v>
       </x:c>
       <x:c r="G115" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="28" customHeight="1">
@@ -3017,13 +3017,13 @@
         <x:v>Paradise Valley</x:v>
       </x:c>
       <x:c r="E116" s="14" t="str">
-        <x:v>The Sparring Grounds</x:v>
+        <x:v>The Sparring Ground</x:v>
       </x:c>
       <x:c r="F116" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #216, Topic 392); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G116" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="28" customHeight="1">
@@ -3037,13 +3037,13 @@
         <x:v>Bernard Jacobs</x:v>
       </x:c>
       <x:c r="D117" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E117" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F117" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #806, Topic 1559).</x:v>
       </x:c>
       <x:c r="G117" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3066,7 +3066,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F118" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #932, Topic 1559).</x:v>
       </x:c>
       <x:c r="G118" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3089,7 +3089,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F119" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #996, Topic 1560).</x:v>
       </x:c>
       <x:c r="G119" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3112,10 +3112,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F120" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G120" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="28" customHeight="1">
@@ -3135,7 +3135,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F121" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #869, Topic 1529).</x:v>
       </x:c>
       <x:c r="G121" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3158,7 +3158,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F122" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #877, Topic 1529).</x:v>
       </x:c>
       <x:c r="G122" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3181,7 +3181,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F123" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #966, Topic 1530).</x:v>
       </x:c>
       <x:c r="G123" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3204,10 +3204,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F124" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G124" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="28" customHeight="1">
@@ -3221,13 +3221,13 @@
         <x:v>Gonzalo Ramirez</x:v>
       </x:c>
       <x:c r="D125" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E125" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F125" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #845, Topic 1521).</x:v>
       </x:c>
       <x:c r="G125" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3250,7 +3250,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F126" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1012, Topic 1521).</x:v>
       </x:c>
       <x:c r="G126" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3273,7 +3273,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F127" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #991, Topic 1522).</x:v>
       </x:c>
       <x:c r="G127" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3296,10 +3296,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F128" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G128" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="28" customHeight="1">
@@ -3319,7 +3319,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F129" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #954, Topic 1545).</x:v>
       </x:c>
       <x:c r="G129" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3342,7 +3342,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F130" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #868, Topic 1545).</x:v>
       </x:c>
       <x:c r="G130" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3365,7 +3365,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F131" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #923, Topic 1546).</x:v>
       </x:c>
       <x:c r="G131" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3388,10 +3388,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F132" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G132" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="28" customHeight="1">
@@ -3405,13 +3405,13 @@
         <x:v>Calvin Black</x:v>
       </x:c>
       <x:c r="D133" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E133" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F133" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #816, Topic 1513).</x:v>
       </x:c>
       <x:c r="G133" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3434,7 +3434,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F134" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #825, Topic 1513).</x:v>
       </x:c>
       <x:c r="G134" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3457,7 +3457,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F135" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1043, Topic 1514).</x:v>
       </x:c>
       <x:c r="G135" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3480,10 +3480,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F136" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G136" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="28" customHeight="1">
@@ -3503,7 +3503,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F137" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #805, Topic 1515).</x:v>
       </x:c>
       <x:c r="G137" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3526,7 +3526,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F138" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #833, Topic 1515).</x:v>
       </x:c>
       <x:c r="G138" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3549,7 +3549,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F139" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #837, Topic 1516).</x:v>
       </x:c>
       <x:c r="G139" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3572,10 +3572,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F140" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G140" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="28" customHeight="1">
@@ -3595,10 +3595,10 @@
         <x:v>Buccaneers' Lair</x:v>
       </x:c>
       <x:c r="F141" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #533, Topic 399); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G141" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="28" customHeight="1">
@@ -3618,10 +3618,10 @@
         <x:v>Smugglers' Guild</x:v>
       </x:c>
       <x:c r="F142" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #534, Topic 400); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G142" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="28" customHeight="1">
@@ -3641,10 +3641,10 @@
         <x:v>Smugglers' Guild</x:v>
       </x:c>
       <x:c r="F143" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; MAW-PDF: Meister auch GM.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen. Echter GM-Lehrer: siehe Paradise Valley (nächste Zeile).</x:v>
       </x:c>
       <x:c r="G143" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="28" customHeight="1">
@@ -3661,13 +3661,13 @@
         <x:v>Paradise Valley</x:v>
       </x:c>
       <x:c r="E144" s="14" t="str">
-        <x:v>The Sparring Grounds</x:v>
+        <x:v>The Sparring Ground</x:v>
       </x:c>
       <x:c r="F144" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #535, Topic 401); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G144" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="28" customHeight="1">
@@ -3687,10 +3687,10 @@
         <x:v>Blades' End</x:v>
       </x:c>
       <x:c r="F145" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #172, Topic 366); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G145" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="146" ht="28" customHeight="1">
@@ -3710,10 +3710,10 @@
         <x:v>Duelists' Edge</x:v>
       </x:c>
       <x:c r="F146" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #173, Topic 367); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G146" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="147" ht="28" customHeight="1">
@@ -3733,10 +3733,10 @@
         <x:v>Duelists' Edge</x:v>
       </x:c>
       <x:c r="F147" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; MAW-PDF: Meister auch GM.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen. Echter GM-Lehrer: siehe Paradise Valley (nächste Zeile).</x:v>
       </x:c>
       <x:c r="G147" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="148" ht="28" customHeight="1">
@@ -3753,13 +3753,13 @@
         <x:v>Paradise Valley</x:v>
       </x:c>
       <x:c r="E148" s="14" t="str">
-        <x:v>Tavern</x:v>
+        <x:v>The Last Chance (Taverne)</x:v>
       </x:c>
       <x:c r="F148" s="14" t="str">
-        <x:v>MAW-Lua bestätigt Ort; Gebäude laut MAW-PDF.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #174, Topic 368); verschoben per zzMAW_MoveTrainers.lua.</x:v>
       </x:c>
       <x:c r="G148" s="18" t="str">
-        <x:v>Lua 4.5 + PDF</x:v>
+        <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="149" ht="28" customHeight="1">
@@ -3779,7 +3779,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F149" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #1008, Topic 1541).</x:v>
       </x:c>
       <x:c r="G149" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3802,7 +3802,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F150" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #879, Topic 1541).</x:v>
       </x:c>
       <x:c r="G150" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3819,13 +3819,13 @@
         <x:v>Harper Collins</x:v>
       </x:c>
       <x:c r="D151" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E151" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F151" s="14" t="str">
-        <x:v>Ältere MMMerge-Angabe; nicht mit MAW 4.5 bestätigt.</x:v>
+        <x:v>Mit Spieldaten abgeglichen (NPC #829, Topic 1542).</x:v>
       </x:c>
       <x:c r="G151" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
@@ -3842,16 +3842,16 @@
         <x:v>Harper Collins</x:v>
       </x:c>
       <x:c r="D152" s="22" t="str">
-        <x:v>Mist</x:v>
+        <x:v>Mist (Misty Islands)</x:v>
       </x:c>
       <x:c r="E152" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F152" s="14" t="str">
-        <x:v>MM6-Meister laut MAW-PDF auch Großmeister; Name ungeprüft.</x:v>
+        <x:v>Nur laut MAW-PDF (Enroth-Meister auch GM). NPC hat in den Spieldaten kein GM-Topic – im Spiel prüfen.</x:v>
       </x:c>
       <x:c r="G152" s="22" t="str">
-        <x:v>MAW-PDF + NPCData</x:v>
+        <x:v>MAW-PDF 4.5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3865,11 +3865,11 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="Rb1a3a0ba5d484d8d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="R8facdfedb9f340df"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="Rf4a7c61f99c14704"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="Ree18af744fd24df1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="Rf45792f913014461"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Re6ca28713b3f4c1b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="R6e87a446cc6c417d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R77f1fcb6d0204900"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="Ree18af744fd24df1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="R960b944749904cbe"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="Refa59963a71a42db"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="Rd9ea746849d24ac8"/>
@@ -3879,11 +3879,11 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="Rff9618d2c3194878"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="Rb54a8ec9c8574069"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="R3e89dfac1322448c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Rcfbaf9ad8833451e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Ree18af744fd24df1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="R87ca6b7e7afe46a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="Rcc707001c3e14224"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="Ree18af744fd24df1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="R3a70e04d8c434ec9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Rbde5d05040ef4be6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Ree18af744fd24df1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="R2e64b176329f4e3f"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R8a5e90faad0b43c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="Rd329eb59098a43eb"/>
@@ -3891,7 +3891,7 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="Red22568290bc41ed"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="Re7ec49ef59e64fb6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="R0267e09aa89d480a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="R6c8adf490f544d0e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="R0921ec36a401407d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Rc5abdf9756e348c4"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="Ra779972afe094145"/>
@@ -3947,7 +3947,7 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="Rd169b3c42a494266"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="R22fe5a0d6af548bc"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="Re0506a20bef7447d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="Re0f26e731f394356"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="R96ecee4d96e34beb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="Reeb56d8305f4485a"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="Rc05d8ef787bd498f"/>
@@ -3971,7 +3971,7 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="R90bb8b9a7d4d4f2e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="R7a664dfa3f1e4457"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="R1be5b9152eda4cf4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="R9616a2dd270446da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="R63fdd86f68f64ddb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="Rfcaf88ece6d14034"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="R1b9d28312ad043ff"/>
@@ -3979,7 +3979,7 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="R1dbb9e84e5c64c6c"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R964d2c381f974eba"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="Rdff07db4a7994f0f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R82775a65c5f74b88"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="R55c77f686cce49b2"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R26a3dadef8954f3a"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="Rdff14d64b6334f15"/>
@@ -4011,7 +4011,7 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="R3d971234698b4b75"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="R667ebf99ca214fbe"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="R2f3f591b73c64f49"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="R04bd95f220d94dc1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="R963182ffbd004242"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="Rdacf220d5676400b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="Rc148edd36d5340c2"/>
@@ -4083,7 +4083,7 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="Rf14fad59f1974bb1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="R2c4062d1ffe443cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="Rae71202d5e3c4fbb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="Rfdf685137fea4c11"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="R56f85c097fe043ce"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G116" r:id="Rfb9e865e3ed24f1d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="Rb4eb21515b864a30"/>
@@ -4139,7 +4139,7 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="R9b47447901ad4bad"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G142" r:id="R0bd8a019570a4c8d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="Ra7c8428631e042f0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G143" r:id="R126ec369f36147e4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G143" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="R5578af195bf843ab"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G144" r:id="R28600764bece40c7"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="R1ca4687e72cc45b7"/>
@@ -4147,7 +4147,7 @@
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="Rd390416b78b64058"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G146" r:id="Rbb251541e20a4d44"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="Rb1ce24b9409241f3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="R5cfa0f3aa9454dd5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="Rc1f71d23eac04ca9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="Rceda730e3fb94b3b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G148" r:id="R4a96a856110c4740"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="R5f2275543dd24a3d"/>

</xml_diff>

<commit_message>
Add Fandom map links to trainer list
Two new columns: a link to the Might and Magic Wiki (Fandom) town page
with its numbered map guide, and the building number of the teacher on
that map (126 of 151 rows; the rest link only, where the wiki places
the teacher outside the town map or differs from MMMerge data).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAW_Guidebook/MAW_MMMerge_4_5_Trainerliste_V3.xlsx
+++ b/MAW_Guidebook/MAW_MMMerge_4_5_Trainerliste_V3.xlsx
@@ -140,8 +140,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MAWTrainerMM6" displayName="MAWTrainerMM6" ref="A1:G152" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="7">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MAWTrainerMM6" displayName="MAWTrainerMM6" ref="A1:I152" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
     <x:tableColumn id="1" name="Fähigkeit"/>
     <x:tableColumn id="2" name="Rang"/>
     <x:tableColumn id="3" name="Trainername"/>
@@ -149,6 +149,8 @@
     <x:tableColumn id="5" name="Haus"/>
     <x:tableColumn id="6" name="Anmerkung"/>
     <x:tableColumn id="7" name="Quelle"/>
+    <x:tableColumn id="8" name="Karte (Fandom)"/>
+    <x:tableColumn id="9" name="Nr. auf Karte"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -356,6 +358,8 @@
     <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="85" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -380,6 +384,12 @@
       <x:c r="G1" s="4" t="str">
         <x:v>Quelle</x:v>
       </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>Karte (Fandom)</x:v>
+      </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>Nr. auf Karte</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="14" t="str">
@@ -403,6 +413,12 @@
       <x:c r="G2" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H2" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I2" s="14" t="str">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -426,6 +442,12 @@
       <x:c r="G3" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H3" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I3" s="14" t="str">
+        <x:v>17</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -449,6 +471,12 @@
       <x:c r="G4" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H4" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I4" s="14" t="str">
+        <x:v>25</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="14" t="str">
@@ -472,6 +500,12 @@
       <x:c r="G5" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H5" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I5" s="14" t="str">
+        <x:v>25</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="14" t="str">
@@ -495,6 +529,12 @@
       <x:c r="G6" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H6" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I6" s="14" t="str">
+        <x:v>8</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="14" t="str">
@@ -518,6 +558,12 @@
       <x:c r="G7" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H7" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I7" s="14" t="str">
+        <x:v>44</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="14" t="str">
@@ -541,6 +587,12 @@
       <x:c r="G8" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H8" s="22" t="str">
+        <x:v>Fandom: Frozen Highlands</x:v>
+      </x:c>
+      <x:c r="I8" s="14" t="str">
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="14" t="str">
@@ -564,6 +616,12 @@
       <x:c r="G9" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H9" s="22" t="str">
+        <x:v>Fandom: Frozen Highlands</x:v>
+      </x:c>
+      <x:c r="I9" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="14" t="str">
@@ -587,6 +645,12 @@
       <x:c r="G10" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H10" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I10" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="14" t="str">
@@ -610,6 +674,12 @@
       <x:c r="G11" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H11" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I11" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="14" t="str">
@@ -633,6 +703,12 @@
       <x:c r="G12" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H12" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I12" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="14" t="str">
@@ -656,6 +732,12 @@
       <x:c r="G13" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H13" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I13" s="14" t="str">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="14" t="str">
@@ -679,6 +761,12 @@
       <x:c r="G14" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H14" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I14" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="14" t="str">
@@ -702,6 +790,12 @@
       <x:c r="G15" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H15" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I15" s="14" t="str">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="14" t="str">
@@ -725,6 +819,12 @@
       <x:c r="G16" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H16" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I16" s="14" t="str">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="14" t="str">
@@ -748,6 +848,12 @@
       <x:c r="G17" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H17" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I17" s="14" t="str">
+        <x:v>19</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="14" t="str">
@@ -771,6 +877,12 @@
       <x:c r="G18" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H18" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I18" s="14" t="str">
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="14" t="str">
@@ -794,6 +906,12 @@
       <x:c r="G19" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H19" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I19" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="14" t="str">
@@ -817,6 +935,12 @@
       <x:c r="G20" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H20" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I20" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="14" t="str">
@@ -840,6 +964,12 @@
       <x:c r="G21" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H21" s="22" t="str">
+        <x:v>Fandom: Alamos</x:v>
+      </x:c>
+      <x:c r="I21" s="14" t="str">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="14" t="str">
@@ -863,6 +993,12 @@
       <x:c r="G22" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H22" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I22" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="14" t="str">
@@ -886,6 +1022,12 @@
       <x:c r="G23" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H23" s="22" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I23" s="14" t="str">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="14" t="str">
@@ -909,6 +1051,12 @@
       <x:c r="G24" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H24" s="22" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I24" s="14" t="str">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="14" t="str">
@@ -932,6 +1080,12 @@
       <x:c r="G25" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H25" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I25" s="14" t="str">
+        <x:v>76</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="14" t="str">
@@ -955,6 +1109,12 @@
       <x:c r="G26" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H26" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I26" s="14" t="str">
+        <x:v>24</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="14" t="str">
@@ -978,6 +1138,12 @@
       <x:c r="G27" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H27" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I27" s="14" t="str">
+        <x:v>62</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="14" t="str">
@@ -1001,6 +1167,12 @@
       <x:c r="G28" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H28" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I28" s="14" t="str">
+        <x:v>62</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="14" t="str">
@@ -1024,6 +1196,12 @@
       <x:c r="G29" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H29" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I29" s="14" t="str">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="14" t="str">
@@ -1047,6 +1225,12 @@
       <x:c r="G30" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H30" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I30" s="14" t="str">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="14" t="str">
@@ -1070,6 +1254,12 @@
       <x:c r="G31" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H31" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I31" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="14" t="str">
@@ -1093,6 +1283,12 @@
       <x:c r="G32" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H32" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I32" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="14" t="str">
@@ -1116,6 +1312,12 @@
       <x:c r="G33" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H33" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I33" s="14" t="str">
+        <x:v>25</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="14" t="str">
@@ -1139,6 +1341,12 @@
       <x:c r="G34" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H34" s="22" t="str">
+        <x:v>Fandom: Frozen Highlands</x:v>
+      </x:c>
+      <x:c r="I34" s="14" t="str">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="14" t="str">
@@ -1162,6 +1370,12 @@
       <x:c r="G35" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H35" s="22" t="str">
+        <x:v>Fandom: Kriegspire</x:v>
+      </x:c>
+      <x:c r="I35" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="14" t="str">
@@ -1185,6 +1399,12 @@
       <x:c r="G36" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H36" s="22" t="str">
+        <x:v>Fandom: Kriegspire</x:v>
+      </x:c>
+      <x:c r="I36" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="14" t="str">
@@ -1208,6 +1428,12 @@
       <x:c r="G37" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H37" s="22" t="str">
+        <x:v>Fandom: Harecksburg</x:v>
+      </x:c>
+      <x:c r="I37" s="14" t="str">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="14" t="str">
@@ -1231,6 +1457,12 @@
       <x:c r="G38" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H38" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I38" s="14" t="str">
+        <x:v>34</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="14" t="str">
@@ -1254,6 +1486,12 @@
       <x:c r="G39" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H39" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I39" s="14" t="str">
+        <x:v>11</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="14" t="str">
@@ -1277,6 +1515,12 @@
       <x:c r="G40" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H40" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I40" s="14" t="str">
+        <x:v>11</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="14" t="str">
@@ -1300,6 +1544,12 @@
       <x:c r="G41" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H41" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I41" s="14" t="str">
+        <x:v>23</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="14" t="str">
@@ -1323,6 +1573,12 @@
       <x:c r="G42" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H42" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I42" s="14" t="str">
+        <x:v>49</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="14" t="str">
@@ -1346,6 +1602,12 @@
       <x:c r="G43" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H43" s="22" t="str">
+        <x:v>Fandom: Hargraeve</x:v>
+      </x:c>
+      <x:c r="I43" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="14" t="str">
@@ -1369,6 +1631,12 @@
       <x:c r="G44" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H44" s="22" t="str">
+        <x:v>Fandom: Hargraeve</x:v>
+      </x:c>
+      <x:c r="I44" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="25" t="str">
@@ -1392,6 +1660,12 @@
       <x:c r="G45" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H45" s="18" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I45" s="14" t="str">
+        <x:v>15</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="25" t="str">
@@ -1415,6 +1689,12 @@
       <x:c r="G46" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H46" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I46" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="25" t="str">
@@ -1438,6 +1718,12 @@
       <x:c r="G47" s="18" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H47" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I47" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="25" t="str">
@@ -1461,6 +1747,12 @@
       <x:c r="G48" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H48" s="18" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I48" s="14" t="str">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="14" t="str">
@@ -1484,6 +1776,12 @@
       <x:c r="G49" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H49" s="22" t="str">
+        <x:v>Fandom: Blackshire</x:v>
+      </x:c>
+      <x:c r="I49" s="14" t="str">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="14" t="str">
@@ -1507,6 +1805,12 @@
       <x:c r="G50" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H50" s="22" t="str">
+        <x:v>Fandom: White Cap</x:v>
+      </x:c>
+      <x:c r="I50" s="14" t="str">
+        <x:v>16</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="14" t="str">
@@ -1530,6 +1834,12 @@
       <x:c r="G51" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H51" s="22" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I51" s="14" t="str">
+        <x:v>22</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="14" t="str">
@@ -1553,6 +1863,12 @@
       <x:c r="G52" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H52" s="22" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I52" s="14" t="str">
+        <x:v>22</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="14" t="str">
@@ -1576,6 +1892,12 @@
       <x:c r="G53" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H53" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I53" s="14" t="str">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="14" t="str">
@@ -1599,6 +1921,12 @@
       <x:c r="G54" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H54" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I54" s="14" t="str">
+        <x:v>15</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="14" t="str">
@@ -1622,6 +1950,12 @@
       <x:c r="G55" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H55" s="22" t="str">
+        <x:v>Fandom: Hargraeve</x:v>
+      </x:c>
+      <x:c r="I55" s="14" t="str">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="14" t="str">
@@ -1645,6 +1979,12 @@
       <x:c r="G56" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H56" s="22" t="str">
+        <x:v>Fandom: Hargraeve</x:v>
+      </x:c>
+      <x:c r="I56" s="14" t="str">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="25" t="str">
@@ -1668,6 +2008,12 @@
       <x:c r="G57" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H57" s="18" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I57" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="25" t="str">
@@ -1691,6 +2037,12 @@
       <x:c r="G58" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H58" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I58" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="25" t="str">
@@ -1714,6 +2066,12 @@
       <x:c r="G59" s="18" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H59" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I59" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="25" t="str">
@@ -1737,6 +2095,12 @@
       <x:c r="G60" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H60" s="18" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I60" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="25" t="str">
@@ -1760,6 +2124,12 @@
       <x:c r="G61" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H61" s="18" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I61" s="14" t="str">
+        <x:v>15</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="25" t="str">
@@ -1783,6 +2153,12 @@
       <x:c r="G62" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H62" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I62" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="25" t="str">
@@ -1806,6 +2182,12 @@
       <x:c r="G63" s="18" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H63" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I63" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="25" t="str">
@@ -1829,6 +2211,12 @@
       <x:c r="G64" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H64" s="18" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I64" s="14" t="str">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="14" t="str">
@@ -1852,6 +2240,12 @@
       <x:c r="G65" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H65" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I65" s="14" t="str">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="14" t="str">
@@ -1875,6 +2269,12 @@
       <x:c r="G66" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H66" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I66" s="14" t="str">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="14" t="str">
@@ -1898,6 +2298,12 @@
       <x:c r="G67" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H67" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I67" s="14" t="str">
+        <x:v>54</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="14" t="str">
@@ -1921,6 +2327,12 @@
       <x:c r="G68" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H68" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I68" s="14" t="str">
+        <x:v>54</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="14" t="str">
@@ -1944,6 +2356,12 @@
       <x:c r="G69" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H69" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I69" s="14" t="str">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="14" t="str">
@@ -1967,6 +2385,12 @@
       <x:c r="G70" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H70" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I70" s="14" t="str">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="14" t="str">
@@ -1990,6 +2414,12 @@
       <x:c r="G71" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H71" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I71" s="14" t="str">
+        <x:v>26</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="14" t="str">
@@ -2013,6 +2443,12 @@
       <x:c r="G72" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H72" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I72" s="14" t="str">
+        <x:v>26</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="14" t="str">
@@ -2036,6 +2472,12 @@
       <x:c r="G73" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H73" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I73" s="14" t="str">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="14" t="str">
@@ -2059,6 +2501,12 @@
       <x:c r="G74" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H74" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I74" s="14" t="str">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="14" t="str">
@@ -2082,6 +2530,12 @@
       <x:c r="G75" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H75" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I75" s="14" t="str">
+        <x:v>59</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="14" t="str">
@@ -2105,6 +2559,12 @@
       <x:c r="G76" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H76" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I76" s="14" t="str">
+        <x:v>59</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="25" t="str">
@@ -2128,6 +2588,12 @@
       <x:c r="G77" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H77" s="18" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I77" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="25" t="str">
@@ -2151,6 +2617,12 @@
       <x:c r="G78" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H78" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I78" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="25" t="str">
@@ -2174,6 +2646,12 @@
       <x:c r="G79" s="18" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H79" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I79" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="25" t="str">
@@ -2197,6 +2675,12 @@
       <x:c r="G80" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H80" s="18" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I80" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="14" t="str">
@@ -2220,6 +2704,12 @@
       <x:c r="G81" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H81" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I81" s="14" t="str">
+        <x:v>32</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="14" t="str">
@@ -2243,6 +2733,12 @@
       <x:c r="G82" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H82" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I82" s="14" t="str">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="14" t="str">
@@ -2266,6 +2762,12 @@
       <x:c r="G83" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H83" s="22" t="str">
+        <x:v>Fandom: Hargraeve</x:v>
+      </x:c>
+      <x:c r="I83" s="14" t="str">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="14" t="str">
@@ -2289,6 +2791,12 @@
       <x:c r="G84" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H84" s="22" t="str">
+        <x:v>Fandom: Hargraeve</x:v>
+      </x:c>
+      <x:c r="I84" s="14" t="str">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="14" t="str">
@@ -2312,6 +2820,12 @@
       <x:c r="G85" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H85" s="22" t="str">
+        <x:v>Fandom: Kriegspire</x:v>
+      </x:c>
+      <x:c r="I85" s="14" t="str">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="14" t="str">
@@ -2335,6 +2849,12 @@
       <x:c r="G86" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H86" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I86" s="14" t="str">
+        <x:v>60</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="14" t="str">
@@ -2358,6 +2878,12 @@
       <x:c r="G87" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H87" s="22" t="str">
+        <x:v>Fandom: Eel-infested Waters</x:v>
+      </x:c>
+      <x:c r="I87" s="14" t="str">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="14" t="str">
@@ -2381,6 +2907,12 @@
       <x:c r="G88" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H88" s="22" t="str">
+        <x:v>Fandom: Eel-infested Waters</x:v>
+      </x:c>
+      <x:c r="I88" s="14" t="str">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="14" t="str">
@@ -2404,6 +2936,12 @@
       <x:c r="G89" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H89" s="22" t="str">
+        <x:v>Fandom: Frozen Highlands</x:v>
+      </x:c>
+      <x:c r="I89" s="14" t="str">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="14" t="str">
@@ -2427,6 +2965,12 @@
       <x:c r="G90" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H90" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I90" s="14" t="str">
+        <x:v>19</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="14" t="str">
@@ -2450,6 +2994,12 @@
       <x:c r="G91" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H91" s="22" t="str">
+        <x:v>Fandom: Blackshire</x:v>
+      </x:c>
+      <x:c r="I91" s="14" t="str">
+        <x:v>26</x:v>
+      </x:c>
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="14" t="str">
@@ -2473,6 +3023,12 @@
       <x:c r="G92" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H92" s="22" t="str">
+        <x:v>Fandom: Blackshire</x:v>
+      </x:c>
+      <x:c r="I92" s="14" t="str">
+        <x:v>26</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="14" t="str">
@@ -2496,6 +3052,12 @@
       <x:c r="G93" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H93" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I93" s="14" t="str">
+        <x:v>16</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="14" t="str">
@@ -2519,6 +3081,12 @@
       <x:c r="G94" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H94" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I94" s="14" t="str">
+        <x:v>47</x:v>
+      </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="14" t="str">
@@ -2542,6 +3110,12 @@
       <x:c r="G95" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H95" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I95" s="14" t="str">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="14" t="str">
@@ -2565,6 +3139,12 @@
       <x:c r="G96" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H96" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I96" s="14" t="str">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="14" t="str">
@@ -2588,6 +3168,12 @@
       <x:c r="G97" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H97" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I97" s="14" t="str">
+        <x:v>43</x:v>
+      </x:c>
     </x:row>
     <x:row r="98" ht="28" customHeight="1">
       <x:c r="A98" s="14" t="str">
@@ -2611,6 +3197,12 @@
       <x:c r="G98" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H98" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I98" s="14" t="str">
+        <x:v>5 / 30</x:v>
+      </x:c>
     </x:row>
     <x:row r="99" ht="28" customHeight="1">
       <x:c r="A99" s="14" t="str">
@@ -2634,6 +3226,12 @@
       <x:c r="G99" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H99" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I99" s="14" t="str">
+        <x:v>46</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" ht="28" customHeight="1">
       <x:c r="A100" s="14" t="str">
@@ -2657,6 +3255,12 @@
       <x:c r="G100" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H100" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I100" s="14" t="str">
+        <x:v>46</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="28" customHeight="1">
       <x:c r="A101" s="14" t="str">
@@ -2680,6 +3284,12 @@
       <x:c r="G101" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H101" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I101" s="14" t="str">
+        <x:v>74</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" ht="28" customHeight="1">
       <x:c r="A102" s="14" t="str">
@@ -2703,6 +3313,12 @@
       <x:c r="G102" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H102" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I102" s="14" t="str">
+        <x:v>23</x:v>
+      </x:c>
     </x:row>
     <x:row r="103" ht="28" customHeight="1">
       <x:c r="A103" s="14" t="str">
@@ -2726,6 +3342,12 @@
       <x:c r="G103" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H103" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I103" s="14" t="str">
+        <x:v>63</x:v>
+      </x:c>
     </x:row>
     <x:row r="104" ht="28" customHeight="1">
       <x:c r="A104" s="14" t="str">
@@ -2749,6 +3371,12 @@
       <x:c r="G104" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H104" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I104" s="14" t="str">
+        <x:v>63</x:v>
+      </x:c>
     </x:row>
     <x:row r="105" ht="28" customHeight="1">
       <x:c r="A105" s="14" t="str">
@@ -2772,6 +3400,12 @@
       <x:c r="G105" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H105" s="22" t="str">
+        <x:v>Fandom: Harecksburg</x:v>
+      </x:c>
+      <x:c r="I105" s="14" t="str">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="106" ht="28" customHeight="1">
       <x:c r="A106" s="14" t="str">
@@ -2795,6 +3429,12 @@
       <x:c r="G106" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H106" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I106" s="14" t="str">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="107" ht="28" customHeight="1">
       <x:c r="A107" s="14" t="str">
@@ -2818,6 +3458,12 @@
       <x:c r="G107" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H107" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I107" s="14" t="str">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="108" ht="28" customHeight="1">
       <x:c r="A108" s="14" t="str">
@@ -2841,6 +3487,12 @@
       <x:c r="G108" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H108" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I108" s="14" t="str">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="109" ht="28" customHeight="1">
       <x:c r="A109" s="14" t="str">
@@ -2864,6 +3516,12 @@
       <x:c r="G109" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H109" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I109" s="14" t="str">
+        <x:v>33</x:v>
+      </x:c>
     </x:row>
     <x:row r="110" ht="28" customHeight="1">
       <x:c r="A110" s="14" t="str">
@@ -2887,6 +3545,12 @@
       <x:c r="G110" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H110" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I110" s="14" t="str">
+        <x:v>17</x:v>
+      </x:c>
     </x:row>
     <x:row r="111" ht="28" customHeight="1">
       <x:c r="A111" s="14" t="str">
@@ -2910,6 +3574,12 @@
       <x:c r="G111" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H111" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I111" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="112" ht="28" customHeight="1">
       <x:c r="A112" s="14" t="str">
@@ -2933,6 +3603,12 @@
       <x:c r="G112" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H112" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I112" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="113" ht="28" customHeight="1">
       <x:c r="A113" s="25" t="str">
@@ -2956,6 +3632,12 @@
       <x:c r="G113" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H113" s="18" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I113" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="28" customHeight="1">
       <x:c r="A114" s="25" t="str">
@@ -2979,6 +3661,12 @@
       <x:c r="G114" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H114" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I114" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="115" ht="28" customHeight="1">
       <x:c r="A115" s="25" t="str">
@@ -3002,6 +3690,12 @@
       <x:c r="G115" s="18" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H115" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I115" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="116" ht="28" customHeight="1">
       <x:c r="A116" s="25" t="str">
@@ -3025,6 +3719,12 @@
       <x:c r="G116" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H116" s="18" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I116" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="117" ht="28" customHeight="1">
       <x:c r="A117" s="14" t="str">
@@ -3048,6 +3748,12 @@
       <x:c r="G117" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H117" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I117" s="14" t="str">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="118" ht="28" customHeight="1">
       <x:c r="A118" s="14" t="str">
@@ -3071,6 +3777,12 @@
       <x:c r="G118" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H118" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I118" s="14" t="str">
+        <x:v>23</x:v>
+      </x:c>
     </x:row>
     <x:row r="119" ht="28" customHeight="1">
       <x:c r="A119" s="14" t="str">
@@ -3094,6 +3806,12 @@
       <x:c r="G119" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H119" s="22" t="str">
+        <x:v>Fandom: Hargraeve</x:v>
+      </x:c>
+      <x:c r="I119" s="14" t="str">
+        <x:v>17</x:v>
+      </x:c>
     </x:row>
     <x:row r="120" ht="28" customHeight="1">
       <x:c r="A120" s="14" t="str">
@@ -3117,6 +3835,12 @@
       <x:c r="G120" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H120" s="22" t="str">
+        <x:v>Fandom: Hargraeve</x:v>
+      </x:c>
+      <x:c r="I120" s="14" t="str">
+        <x:v>17</x:v>
+      </x:c>
     </x:row>
     <x:row r="121" ht="28" customHeight="1">
       <x:c r="A121" s="14" t="str">
@@ -3140,6 +3864,12 @@
       <x:c r="G121" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H121" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I121" s="14" t="str">
+        <x:v>31</x:v>
+      </x:c>
     </x:row>
     <x:row r="122" ht="28" customHeight="1">
       <x:c r="A122" s="14" t="str">
@@ -3163,6 +3893,12 @@
       <x:c r="G122" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H122" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I122" s="14" t="str">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="123" ht="28" customHeight="1">
       <x:c r="A123" s="14" t="str">
@@ -3186,6 +3922,12 @@
       <x:c r="G123" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H123" s="22" t="str">
+        <x:v>Fandom: Blackshire</x:v>
+      </x:c>
+      <x:c r="I123" s="14" t="str">
+        <x:v>28</x:v>
+      </x:c>
     </x:row>
     <x:row r="124" ht="28" customHeight="1">
       <x:c r="A124" s="14" t="str">
@@ -3209,6 +3951,12 @@
       <x:c r="G124" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H124" s="22" t="str">
+        <x:v>Fandom: Blackshire</x:v>
+      </x:c>
+      <x:c r="I124" s="14" t="str">
+        <x:v>28</x:v>
+      </x:c>
     </x:row>
     <x:row r="125" ht="28" customHeight="1">
       <x:c r="A125" s="14" t="str">
@@ -3232,6 +3980,12 @@
       <x:c r="G125" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H125" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I125" s="14" t="str">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="126" ht="28" customHeight="1">
       <x:c r="A126" s="14" t="str">
@@ -3255,6 +4009,12 @@
       <x:c r="G126" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H126" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I126" s="14" t="str">
+        <x:v>33</x:v>
+      </x:c>
     </x:row>
     <x:row r="127" ht="28" customHeight="1">
       <x:c r="A127" s="14" t="str">
@@ -3278,6 +4038,12 @@
       <x:c r="G127" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H127" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I127" s="14" t="str">
+        <x:v>23</x:v>
+      </x:c>
     </x:row>
     <x:row r="128" ht="28" customHeight="1">
       <x:c r="A128" s="14" t="str">
@@ -3301,6 +4067,12 @@
       <x:c r="G128" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H128" s="22" t="str">
+        <x:v>Fandom: Darkmoor</x:v>
+      </x:c>
+      <x:c r="I128" s="14" t="str">
+        <x:v>23</x:v>
+      </x:c>
     </x:row>
     <x:row r="129" ht="28" customHeight="1">
       <x:c r="A129" s="14" t="str">
@@ -3324,6 +4096,12 @@
       <x:c r="G129" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H129" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I129" s="14" t="str">
+        <x:v>76</x:v>
+      </x:c>
     </x:row>
     <x:row r="130" ht="28" customHeight="1">
       <x:c r="A130" s="14" t="str">
@@ -3347,6 +4125,12 @@
       <x:c r="G130" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H130" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I130" s="14" t="str">
+        <x:v>22</x:v>
+      </x:c>
     </x:row>
     <x:row r="131" ht="28" customHeight="1">
       <x:c r="A131" s="14" t="str">
@@ -3370,6 +4154,12 @@
       <x:c r="G131" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H131" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I131" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="132" ht="28" customHeight="1">
       <x:c r="A132" s="14" t="str">
@@ -3393,6 +4183,12 @@
       <x:c r="G132" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H132" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I132" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="133" ht="28" customHeight="1">
       <x:c r="A133" s="14" t="str">
@@ -3416,6 +4212,12 @@
       <x:c r="G133" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H133" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I133" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="134" ht="28" customHeight="1">
       <x:c r="A134" s="14" t="str">
@@ -3439,6 +4241,12 @@
       <x:c r="G134" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H134" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I134" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="135" ht="28" customHeight="1">
       <x:c r="A135" s="14" t="str">
@@ -3462,6 +4270,12 @@
       <x:c r="G135" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H135" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I135" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="136" ht="28" customHeight="1">
       <x:c r="A136" s="14" t="str">
@@ -3485,6 +4299,12 @@
       <x:c r="G136" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H136" s="22" t="str">
+        <x:v>Fandom: Silver Cove</x:v>
+      </x:c>
+      <x:c r="I136" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="137" ht="28" customHeight="1">
       <x:c r="A137" s="14" t="str">
@@ -3508,6 +4328,12 @@
       <x:c r="G137" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H137" s="22" t="str">
+        <x:v>Fandom: Ironfist</x:v>
+      </x:c>
+      <x:c r="I137" s="14" t="str">
+        <x:v>22</x:v>
+      </x:c>
     </x:row>
     <x:row r="138" ht="28" customHeight="1">
       <x:c r="A138" s="14" t="str">
@@ -3531,6 +4357,12 @@
       <x:c r="G138" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H138" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I138" s="14" t="str">
+        <x:v>49</x:v>
+      </x:c>
     </x:row>
     <x:row r="139" ht="28" customHeight="1">
       <x:c r="A139" s="14" t="str">
@@ -3554,6 +4386,12 @@
       <x:c r="G139" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H139" s="22" t="str">
+        <x:v>Fandom: Blackshire</x:v>
+      </x:c>
+      <x:c r="I139" s="14" t="str">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="140" ht="28" customHeight="1">
       <x:c r="A140" s="14" t="str">
@@ -3577,6 +4415,12 @@
       <x:c r="G140" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H140" s="22" t="str">
+        <x:v>Fandom: Blackshire</x:v>
+      </x:c>
+      <x:c r="I140" s="14" t="str">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="141" ht="28" customHeight="1">
       <x:c r="A141" s="25" t="str">
@@ -3600,6 +4444,12 @@
       <x:c r="G141" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H141" s="18" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I141" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="142" ht="28" customHeight="1">
       <x:c r="A142" s="25" t="str">
@@ -3623,6 +4473,12 @@
       <x:c r="G142" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H142" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I142" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="143" ht="28" customHeight="1">
       <x:c r="A143" s="25" t="str">
@@ -3646,6 +4502,12 @@
       <x:c r="G143" s="18" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H143" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I143" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="144" ht="28" customHeight="1">
       <x:c r="A144" s="25" t="str">
@@ -3669,6 +4531,12 @@
       <x:c r="G144" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H144" s="18" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I144" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="145" ht="28" customHeight="1">
       <x:c r="A145" s="25" t="str">
@@ -3692,6 +4560,12 @@
       <x:c r="G145" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H145" s="18" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I145" s="14" t="str">
+        <x:v>15</x:v>
+      </x:c>
     </x:row>
     <x:row r="146" ht="28" customHeight="1">
       <x:c r="A146" s="25" t="str">
@@ -3715,6 +4589,12 @@
       <x:c r="G146" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H146" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I146" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="147" ht="28" customHeight="1">
       <x:c r="A147" s="25" t="str">
@@ -3738,6 +4618,12 @@
       <x:c r="G147" s="18" t="str">
         <x:v>MAW-PDF 4.5</x:v>
       </x:c>
+      <x:c r="H147" s="18" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I147" s="14" t="str">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="148" ht="28" customHeight="1">
       <x:c r="A148" s="25" t="str">
@@ -3761,6 +4647,12 @@
       <x:c r="G148" s="18" t="str">
         <x:v>NPCData + Lua 4.5</x:v>
       </x:c>
+      <x:c r="H148" s="18" t="str">
+        <x:v>Fandom: Edenbrook</x:v>
+      </x:c>
+      <x:c r="I148" s="14" t="str">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="149" ht="28" customHeight="1">
       <x:c r="A149" s="14" t="str">
@@ -3784,6 +4676,12 @@
       <x:c r="G149" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H149" s="22" t="str">
+        <x:v>Fandom: Freehaven</x:v>
+      </x:c>
+      <x:c r="I149" s="14" t="str">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="150" ht="28" customHeight="1">
       <x:c r="A150" s="14" t="str">
@@ -3807,6 +4705,12 @@
       <x:c r="G150" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H150" s="22" t="str">
+        <x:v>Fandom: New Sorpigal</x:v>
+      </x:c>
+      <x:c r="I150" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
     </x:row>
     <x:row r="151" ht="28" customHeight="1">
       <x:c r="A151" s="14" t="str">
@@ -3830,6 +4734,12 @@
       <x:c r="G151" s="22" t="str">
         <x:v>MMMerge-NPCData</x:v>
       </x:c>
+      <x:c r="H151" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I151" s="14" t="str">
+        <x:v>24</x:v>
+      </x:c>
     </x:row>
     <x:row r="152" ht="28" customHeight="1">
       <x:c r="A152" s="14" t="str">
@@ -3852,312 +4762,469 @@
       </x:c>
       <x:c r="G152" s="22" t="str">
         <x:v>MAW-PDF 4.5</x:v>
+      </x:c>
+      <x:c r="H152" s="22" t="str">
+        <x:v>Fandom: Mist</x:v>
+      </x:c>
+      <x:c r="I152" s="14" t="str">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="R466e05f4a8ac4754"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="Ree18af744fd24df1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="Ra8e73a5592434bb4"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="Rb4c54b0d52de46de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="Rff8e9e1882bc49b6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R55d9ce8044e14833"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="Rb1a3a0ba5d484d8d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="R8facdfedb9f340df"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="Ree18af744fd24df1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="Rf45792f913014461"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Re6ca28713b3f4c1b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="R6e87a446cc6c417d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="Ree18af744fd24df1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="Raaad9f82b4569d73"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="R960b944749904cbe"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="Refa59963a71a42db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="Raaad9f82b4569d73"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="Rd9ea746849d24ac8"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="Rbf712286848b4189"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="Re67c00b5b64b41ea"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="Re8124895f44e4067"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="Rff9618d2c3194878"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="Rb54a8ec9c8574069"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="R3e89dfac1322448c"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Ree18af744fd24df1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="R87ca6b7e7afe46a9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="Ree18af744fd24df1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="R3a70e04d8c434ec9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Ree18af744fd24df1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="R2e64b176329f4e3f"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R8a5e90faad0b43c1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="Rd329eb59098a43eb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="Rbd5907e33c504874"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="Red22568290bc41ed"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="Re7ec49ef59e64fb6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="R0267e09aa89d480a"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="R0921ec36a401407d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Rc5abdf9756e348c4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="Ra779972afe094145"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="R74eca572a9c94d7a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="R289ebaf300aea12e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="Rbc2490a48b1546b3"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="R9b58300400504342"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="Rbea1fc16d0ed468c"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R9d26d0da2e15428f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="R6ae1dc0d14b84cde"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="Re862ffe6917a4578"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="R9035b73c55a04a86"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="Rade4a602d1344519"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="R450c4aed5d50456f"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="R1289657fb4144e34"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="Rbb1784dde2304834"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="Rd40b20c631ea4e4a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="R9ea290a7525045a0"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R76c076c78d924dc5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="R4a44da174b2d4de0"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="R8a9cd6ddc1d741f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="Rb458a36afb64478b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R0944bec4871a4ce1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="R8f24b7296c094f49"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="R17947ef6b8b64c7a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="Rbc38b98b0bd04ec9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="Rf07613152cb54ec0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="R0da54a9a59c841ba"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R9fbc12a714744826"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="Rb63b763965ef4a63"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R1a700f34ca014c58"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="Raaad9f82b4569d73"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="R746af38e1b10449e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R3f99543ac0c040a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="Rc05930a38908b009"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="R250307b753d24ff0"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="Raaca945ef4a04246"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="Rc05930a38908b009"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="Rdc75d77ce24d413c"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R9b9fbcdf2b4a42d7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="Rb108e47208591f90"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="R0bc98f97d40d49c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="R04ac4d62a96c4807"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="R9a7ca5eba9cc4274"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="R49aac2d2d72b4195"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="R5a8d73b372f0427c"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="R8c813edbd67448ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="R728181cb3be34ca7"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="Rac88fce4eba34ad6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="Rc805eeeb3cdc44b5"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="R1921ddbb5f7a44ee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="Rc303928fd53f423a"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R65c90939cbb147fd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="Rccf980ac0883d7c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="Ra80c925efefa4d89"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="Rc4787ef62daa42b7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="Rccf980ac0883d7c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="R6f4b3c3961a541fe"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="Rd8f53de592254aa1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="Rd169b3c42a494266"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="R22fe5a0d6af548bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="Re0506a20bef7447d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="R96ecee4d96e34beb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="Reeb56d8305f4485a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="Rc05d8ef787bd498f"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="Rda2202715b9f479c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="Rd6c00ec3b1b437e6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="Rf0e224df1c024df8"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R9cf0b7f5134f48d8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="Rca5d6c4af9a4a264"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="R01a64acd04a24cdd"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="Rb40abb278d3e439b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="R77b3a3fc800942d2"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="R7563e37fc83b4dc0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="R0782de0ecb4146a9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R7ee9d2c8be8a494e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="R08b345b5b19e4231"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="R199d04bb4b1749eb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="R21dbf69f17514b7f"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="R9e9c3de2f5d943fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="Rccf980ac0883d7c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="Rde5e228e35dd4e24"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R35d8c60a158a4d7c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="Rccf980ac0883d7c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="R69020146ad08453e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="Rdfe250254fa54135"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="R90bb8b9a7d4d4f2e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="R7a664dfa3f1e4457"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="R1be5b9152eda4cf4"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="R63fdd86f68f64ddb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="Rfcaf88ece6d14034"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="R1b9d28312ad043ff"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="R94d04c7ac1e64893"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="R1dbb9e84e5c64c6c"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R964d2c381f974eba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="Rdff07db4a7994f0f"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="R55c77f686cce49b2"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R26a3dadef8954f3a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="Rdff14d64b6334f15"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="R7109f41531684ca3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="Rb7cdf9bf361b42a4"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="Ra9299c8226ba4d78"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="Rb9766c18d3574002"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="Rdcf13b059c3d4382"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="Rb9f9ef7152b34a71"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="R92951f8d4d264f43"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="Rb24bdeb4c2094762"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="R2f8f7784d6e6482d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="R8a6f9c79f8214a8b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="R328624cd14f64e82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="Rb668a79bd58245d5"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="R8895bd9324ae4f90"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="Ra7bd03b336914f83"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="R0eb77851a71b47f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="R12b303b80b8747d4"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="R0d8b02da60e5485c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="R8e41d339800842ff"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="Rc6abcefdb30c4cb3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="R2ba2a3f95a664788"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="Rd6254ce9801742cb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="R730279cf0a664504"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="R30b9879bd4ba4fbf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="R554a32aeafea416e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="R307301b471c545ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="R3d971234698b4b75"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="R667ebf99ca214fbe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="R2f3f591b73c64f49"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="R963182ffbd004242"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="Rdacf220d5676400b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="Rc148edd36d5340c2"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="Rf2b41c5829544e12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="Rd556bd75aaa54e11"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="Ra56bdac10d724ce5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="Rffab5ff6ceb14d19"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="Rc663ec0bd9fc422f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="Rccf980ac0883d7c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="R3879ac7c766741b1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="R81f3c17f85e4430c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="Rccf980ac0883d7c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="R17180dc2452141db"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="R1ca5edb914d0400e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="Rc05930a38908b009"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="R7c2eacbd331b459a"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="Ra9a8ea7af4284452"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="Rf9e4dc61ff674c3f"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="R5e7e4de503e745e4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="Ra9218f1eb524a146"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="R2f261c888cc642ef"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="Rb535cbf150674ad4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="Ra9218f1eb524a146"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="Rfbc167e0cb91427b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="Ra1d88fc65d2b4de8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="Raaad9f82b4569d73"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="R7c06ccc22686449a"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="R33d9dd8fa2364b9c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="R5e35bd4b655c4075"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="R879973fb0d9d4566"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="Rd6c00ec3b1b437e6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="Rb529c2e941264899"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="Raefe6f934d004360"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="Rd6c00ec3b1b437e6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="R6d75ad9a836f47bc"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="Reebc84706b0e4d82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="R9bc9b968328b4b69"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="R624a1b3df9d44e83"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="Rcd4be44af7104bef"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="R08bef6c6a5da4ebd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="Rab3e5960fa3a4abb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="R4d791461118b4079"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="Ra054e0fee1544fc9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="R1069f1f5e9744a85"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="R1778e9926c1d4719"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="Rd364b26203904682"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="Rb7a1aee298404ae9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="R2027341ff0964e90"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="R946af645ba9f4edf"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="R4b1a63aa49844114"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="R9b8a0f1ff43846f6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="R793795d5201047eb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="R27f0e8828b3b4043"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="Rbd01deb3eba142e3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="Rcec5ad184a9d49f5"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="R172b9a9b2f264604"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="Rc74baed5f196479a"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="Rc7099c901a4a4b95"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="R58deb577875e4f33"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="Re58a9b1993474dfd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="Rb108e47208591f90"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="Rd8180da064794b2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="Rbc9830b39fa14f12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="R3f9902b33e464f41"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="R74d7695f3f9143bb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="Rf9a89821d82242b3"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="R3744ba997acb4c60"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="R92cc65af17ed4e93"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="R8ec3fc5e5c49428c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="R880883a713c64d1d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="Rc483ac6274a24029"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="R0cd2ef2aa20d4726"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="Rf6cc5846f36a4e5d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="Radd69944618340a1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="R760538d3cb294a68"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="R2a8fc2edb38b40da"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="Rec3d7b24b9a04f48"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="Rf14fad59f1974bb1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="R2c4062d1ffe443cb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="Rae71202d5e3c4fbb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="R56f85c097fe043ce"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G116" r:id="Rfb9e865e3ed24f1d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="Rb4eb21515b864a30"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="R4778e4f0026f49b0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="Rceaeaa7e594a4eaf"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="R23493c2e742447a8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="Rbda3f4e4bddb4182"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G119" r:id="R9749523688214502"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="Rccf980ac0883d7c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="Re5ccca47ea334328"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="R1bf46e0b5d11417c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="Rccf980ac0883d7c1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="R6f12cdd419cf4d86"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G121" r:id="Rc747f97596cb4a57"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="Rbdcaafe9b89942c2"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G122" r:id="R744ed5ef085e4467"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="R87c48ef231dd4ef9"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G123" r:id="Rbdac96bb8bf845d9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="Rd6c00ec3b1b437e6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="R160d8bd68761402b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G124" r:id="R17f3cfa481f24161"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="Rd6c00ec3b1b437e6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="R5d188498274a406e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="R09593a52641243ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="R489c34367168472d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G126" r:id="Rf383ab267b424f34"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="R343600ce2d7c44af"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="Rf87ac77bed7343f2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="Rf7b70858fdc241b6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="R920effbb2dfa4166"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="R357a27e232e9586b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="R8f8ce5048efe4711"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G129" r:id="R56fc1afe69d84351"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="R339cdb8e9b3b4b09"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="R534ca7543b904993"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="R8f4ef9358af24b5e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G131" r:id="Recd53e2b041142fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="R3e572e6a9b8448cc"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G132" r:id="R5bf45dad7d834400"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="R6146dcc323b949b2"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G133" r:id="R9002fa12c2bf4c10"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="R709163dfa1ea491e"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G134" r:id="R5a331b0068994d19"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="R66c63894f3f64f45"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G135" r:id="R5ba9ca447e83480c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="Rf062ed278fe949e5"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="Rddbc10d5b2fa438d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="R08f6f81deda034cb"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="R6d2f3f9a292b4278"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="R900b0005f1914bb8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="Rae53dd1c9fdb7119"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="R937c59a593164359"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G138" r:id="Rdeb68d12e0df4345"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="Re02f0b53c87f4144"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G139" r:id="R452e4e54520849d4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" r:id="Rd6c00ec3b1b437e6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="R7b1c6d4eba014b30"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="R41a7404161594f3c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="Rd6c00ec3b1b437e6"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="R509d71f6f39d4e3f"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G141" r:id="R9623c93ebd244fa6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="R9b47447901ad4bad"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G142" r:id="R0bd8a019570a4c8d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="Ra7c8428631e042f0"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G143" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="R5578af195bf843ab"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G144" r:id="R28600764bece40c7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="R1ca4687e72cc45b7"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G145" r:id="R27a0fd65d3f84332"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H145" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="Rd390416b78b64058"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G146" r:id="Rbb251541e20a4d44"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="Rb1ce24b9409241f3"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="Rc1f71d23eac04ca9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H147" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="Rceda730e3fb94b3b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G148" r:id="R4a96a856110c4740"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H148" r:id="R18e29651c4029f2d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="R5f2275543dd24a3d"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G149" r:id="R0e23cad4b1064000"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H149" r:id="R674fc40be3d81887"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="Rc0e7fad6e806412b"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G150" r:id="R133c36b6e8b3416a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H150" r:id="Rc046267506cd8090"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="Rf80bac66214a40aa"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G151" r:id="R41e8e6a22a28442e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H151" r:id="R6999cf087fbdee27"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="R0ae0bb5b2aa344f4"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G152" r:id="R04dd7602b960467f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H152" r:id="R6999cf087fbdee27"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">

</xml_diff>